<commit_message>
Central slice: Stage 4 engine, results API, map, import tab, QA fixes
</commit_message>
<xml_diff>
--- a/design/templates/generated/Central/BUFFALO_DROUGHT_CEN_V1_upload_template.xlsx
+++ b/design/templates/generated/Central/BUFFALO_DROUGHT_CEN_V1_upload_template.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2020-2025" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-2030" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2021-2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-2030" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEIGHTS" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_META" sheetId="5" state="hidden" r:id="rId5"/>
@@ -152,14 +152,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y40"/>
+  <dimension ref="A1:Z45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -560,12 +560,13 @@
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RAW DATA 2020-2025 - Livestock Sector / Buffalo Farming - Drought - Central Province   [profile BUFFALO_DROUGHT_CEN_V1]   |   Enter RAW values only - the system normalizes.</t>
+          <t>RAW DATA 2021-2025 - Livestock Sector / Buffalo Farming - Drought - Central Province   [profile BUFFALO_DROUGHT_CEN_V1]   |   Enter RAW values only - the system normalizes.</t>
         </is>
       </c>
     </row>
@@ -597,100 +598,105 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>DROUGHT_EVENTS_1974_TO_2022</t>
+          <t>DROUGHT_EVENTS_1974_TO_2004</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>DROUGHT_EVENTS_2005_TO_2022</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>DROUGHT_HAZARD_INDEX</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>OCCURRENCE_WARM_DAYS</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>STANDARD_PRECIPITATION_INDEX</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_FARMERS</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_FARMS</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_MILK_PRODUCTION_FARMS</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_POPULATION</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>LIVESTOCK_FARMERS</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>MITCH_BUFFALOES_DAILY_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>PASTURE_FODDER_EXTENT_ACRE</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>PCT_EXTENSIVE</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>PCT_INTENSIVE</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>PCT_SEMI_INTENSIVE</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>DATA_SOURCE</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
@@ -724,118 +730,124 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>hazard: No. of drought events - 1974 to 2022 (1974-2004, 25%, 2005 -2022, 75%)
-&gt;&gt; fixed window - same value on both period tabs</t>
+          <t>hazard: No. of Drought events - 1974 to 2004 (25%)
+&gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>hazard: No. of Drought events - 2005 -2022 (75%)
+&gt;&gt; enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>hazard: Drought Hazard  Index
 &gt;&gt; fixed window - same value on both period tabs</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>hazard: Occurrence of warm days (TX90p)
 &gt;&gt; fixed window - same value on both period tabs</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>hazard: SPI (Intensity)
 &gt;&gt; fixed window - same value on both period tabs</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>exposure: # of Buffalo Farmers
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>exposure: No. of Buffalo Farms
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>exposure: No.of Buffalo Milk Production Farms
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>exposure: Buffalo Population
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>exposure: Total livestock farmers
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>exposure: Annual Mitch Buffalo Milk Production (l)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>exposure: Daily Mitch Buffaloes Milk Production (l)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>exposure: Mitch Buffalo Monthly Milk Production (l)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>exposure: Pasture &amp; Fodder Extent (Acre)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>exposure: % of Buffalo Farmers from total livestock operators
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>exposure: % Extensive
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr">
+      <c r="V3" s="5" t="inlineStr">
         <is>
           <t>exposure: % Intensive
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="V3" s="5" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>exposure: % livestock farmers from total Agricultural Operators
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr">
+      <c r="X3" s="5" t="inlineStr">
         <is>
           <t>exposure: % Semi Intensive
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="X3" s="5" t="inlineStr">
+      <c r="Y3" s="5" t="inlineStr">
         <is>
           <t>origin of the numbers</t>
         </is>
       </c>
-      <c r="Y3" s="5" t="inlineStr">
+      <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
@@ -858,7 +870,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>2025</v>
@@ -917,12 +929,15 @@
       <c r="W4" s="6" t="n">
         <v>737.5</v>
       </c>
-      <c r="X4" s="6" t="inlineStr">
-        <is>
-          <t>Dept. report 2020-2025</t>
-        </is>
+      <c r="X4" s="6" t="n">
+        <v>775</v>
       </c>
       <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>Dept. report 2021-2025</t>
+        </is>
+      </c>
+      <c r="Z4" s="6" t="inlineStr">
         <is>
           <t>example row</t>
         </is>
@@ -931,7 +946,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>CEN-001</t>
+          <t>KA1</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -945,7 +960,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>2025</v>
@@ -970,11 +985,12 @@
       <c r="W5" s="8" t="n"/>
       <c r="X5" s="8" t="n"/>
       <c r="Y5" s="8" t="n"/>
+      <c r="Z5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>CEN-002</t>
+          <t>KA2</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -988,7 +1004,7 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>2025</v>
@@ -1013,11 +1029,12 @@
       <c r="W6" s="8" t="n"/>
       <c r="X6" s="8" t="n"/>
       <c r="Y6" s="8" t="n"/>
+      <c r="Z6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>CEN-003</t>
+          <t>KA3</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1031,7 +1048,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>2025</v>
@@ -1056,11 +1073,12 @@
       <c r="W7" s="8" t="n"/>
       <c r="X7" s="8" t="n"/>
       <c r="Y7" s="8" t="n"/>
+      <c r="Z7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>CEN-004</t>
+          <t>KA4</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -1074,7 +1092,7 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>2025</v>
@@ -1099,11 +1117,12 @@
       <c r="W8" s="8" t="n"/>
       <c r="X8" s="8" t="n"/>
       <c r="Y8" s="8" t="n"/>
+      <c r="Z8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>CEN-005</t>
+          <t>KA5</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1117,7 +1136,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>2025</v>
@@ -1142,11 +1161,12 @@
       <c r="W9" s="8" t="n"/>
       <c r="X9" s="8" t="n"/>
       <c r="Y9" s="8" t="n"/>
+      <c r="Z9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>CEN-006</t>
+          <t>KA6</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1160,7 +1180,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>2025</v>
@@ -1185,11 +1205,12 @@
       <c r="W10" s="8" t="n"/>
       <c r="X10" s="8" t="n"/>
       <c r="Y10" s="8" t="n"/>
+      <c r="Z10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>CEN-007</t>
+          <t>KA7</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1203,7 +1224,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>2025</v>
@@ -1228,11 +1249,12 @@
       <c r="W11" s="8" t="n"/>
       <c r="X11" s="8" t="n"/>
       <c r="Y11" s="8" t="n"/>
+      <c r="Z11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>CEN-008</t>
+          <t>KA8</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -1246,7 +1268,7 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>2025</v>
@@ -1271,11 +1293,12 @@
       <c r="W12" s="8" t="n"/>
       <c r="X12" s="8" t="n"/>
       <c r="Y12" s="8" t="n"/>
+      <c r="Z12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>CEN-009</t>
+          <t>KA9</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -1289,7 +1312,7 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>2025</v>
@@ -1314,11 +1337,12 @@
       <c r="W13" s="8" t="n"/>
       <c r="X13" s="8" t="n"/>
       <c r="Y13" s="8" t="n"/>
+      <c r="Z13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>CEN-010</t>
+          <t>KA10</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -1332,7 +1356,7 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>2025</v>
@@ -1357,11 +1381,12 @@
       <c r="W14" s="8" t="n"/>
       <c r="X14" s="8" t="n"/>
       <c r="Y14" s="8" t="n"/>
+      <c r="Z14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>CEN-011</t>
+          <t>KA11</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -1375,7 +1400,7 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>2025</v>
@@ -1400,11 +1425,12 @@
       <c r="W15" s="8" t="n"/>
       <c r="X15" s="8" t="n"/>
       <c r="Y15" s="8" t="n"/>
+      <c r="Z15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>CEN-012</t>
+          <t>KA12</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -1418,7 +1444,7 @@
         </is>
       </c>
       <c r="D16" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>2025</v>
@@ -1443,11 +1469,12 @@
       <c r="W16" s="8" t="n"/>
       <c r="X16" s="8" t="n"/>
       <c r="Y16" s="8" t="n"/>
+      <c r="Z16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>CEN-013</t>
+          <t>KA13</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -1461,7 +1488,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>2025</v>
@@ -1486,11 +1513,12 @@
       <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n"/>
       <c r="Y17" s="8" t="n"/>
+      <c r="Z17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>CEN-014</t>
+          <t>KA14</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -1504,7 +1532,7 @@
         </is>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>2025</v>
@@ -1529,11 +1557,12 @@
       <c r="W18" s="8" t="n"/>
       <c r="X18" s="8" t="n"/>
       <c r="Y18" s="8" t="n"/>
+      <c r="Z18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>CEN-015</t>
+          <t>KA15</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1547,7 +1576,7 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>2025</v>
@@ -1572,11 +1601,12 @@
       <c r="W19" s="8" t="n"/>
       <c r="X19" s="8" t="n"/>
       <c r="Y19" s="8" t="n"/>
+      <c r="Z19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>CEN-016</t>
+          <t>KA16</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1590,7 +1620,7 @@
         </is>
       </c>
       <c r="D20" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>2025</v>
@@ -1615,11 +1645,12 @@
       <c r="W20" s="8" t="n"/>
       <c r="X20" s="8" t="n"/>
       <c r="Y20" s="8" t="n"/>
+      <c r="Z20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>CEN-017</t>
+          <t>KA17</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1633,7 +1664,7 @@
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E21" s="7" t="n">
         <v>2025</v>
@@ -1658,11 +1689,12 @@
       <c r="W21" s="8" t="n"/>
       <c r="X21" s="8" t="n"/>
       <c r="Y21" s="8" t="n"/>
+      <c r="Z21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>CEN-018</t>
+          <t>KA18</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1676,7 +1708,7 @@
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E22" s="7" t="n">
         <v>2025</v>
@@ -1701,11 +1733,12 @@
       <c r="W22" s="8" t="n"/>
       <c r="X22" s="8" t="n"/>
       <c r="Y22" s="8" t="n"/>
+      <c r="Z22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>CEN-019</t>
+          <t>KA19</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1719,7 +1752,7 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>2025</v>
@@ -1744,11 +1777,12 @@
       <c r="W23" s="8" t="n"/>
       <c r="X23" s="8" t="n"/>
       <c r="Y23" s="8" t="n"/>
+      <c r="Z23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>CEN-020</t>
+          <t>KA20</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1762,7 +1796,7 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>2025</v>
@@ -1787,11 +1821,12 @@
       <c r="W24" s="8" t="n"/>
       <c r="X24" s="8" t="n"/>
       <c r="Y24" s="8" t="n"/>
+      <c r="Z24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>CEN-021</t>
+          <t>MA1</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1805,7 +1840,7 @@
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>2025</v>
@@ -1830,11 +1865,12 @@
       <c r="W25" s="8" t="n"/>
       <c r="X25" s="8" t="n"/>
       <c r="Y25" s="8" t="n"/>
+      <c r="Z25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>CEN-022</t>
+          <t>MA2</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1848,7 +1884,7 @@
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>2025</v>
@@ -1873,11 +1909,12 @@
       <c r="W26" s="8" t="n"/>
       <c r="X26" s="8" t="n"/>
       <c r="Y26" s="8" t="n"/>
+      <c r="Z26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>CEN-023</t>
+          <t>MA3</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1891,7 +1928,7 @@
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>2025</v>
@@ -1916,11 +1953,12 @@
       <c r="W27" s="8" t="n"/>
       <c r="X27" s="8" t="n"/>
       <c r="Y27" s="8" t="n"/>
+      <c r="Z27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>CEN-024</t>
+          <t>MA4</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1934,7 +1972,7 @@
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>2025</v>
@@ -1959,11 +1997,12 @@
       <c r="W28" s="8" t="n"/>
       <c r="X28" s="8" t="n"/>
       <c r="Y28" s="8" t="n"/>
+      <c r="Z28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>CEN-025</t>
+          <t>MA5</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1977,7 +2016,7 @@
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>2025</v>
@@ -2002,11 +2041,12 @@
       <c r="W29" s="8" t="n"/>
       <c r="X29" s="8" t="n"/>
       <c r="Y29" s="8" t="n"/>
+      <c r="Z29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>CEN-026</t>
+          <t>MA6</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -2020,7 +2060,7 @@
         </is>
       </c>
       <c r="D30" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E30" s="7" t="n">
         <v>2025</v>
@@ -2045,11 +2085,12 @@
       <c r="W30" s="8" t="n"/>
       <c r="X30" s="8" t="n"/>
       <c r="Y30" s="8" t="n"/>
+      <c r="Z30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>CEN-027</t>
+          <t>MA7</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -2063,7 +2104,7 @@
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>2025</v>
@@ -2088,11 +2129,12 @@
       <c r="W31" s="8" t="n"/>
       <c r="X31" s="8" t="n"/>
       <c r="Y31" s="8" t="n"/>
+      <c r="Z31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>CEN-028</t>
+          <t>MA8</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2106,7 +2148,7 @@
         </is>
       </c>
       <c r="D32" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>2025</v>
@@ -2131,11 +2173,12 @@
       <c r="W32" s="8" t="n"/>
       <c r="X32" s="8" t="n"/>
       <c r="Y32" s="8" t="n"/>
+      <c r="Z32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>CEN-029</t>
+          <t>MA9</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2149,7 +2192,7 @@
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>2025</v>
@@ -2174,11 +2217,12 @@
       <c r="W33" s="8" t="n"/>
       <c r="X33" s="8" t="n"/>
       <c r="Y33" s="8" t="n"/>
+      <c r="Z33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>CEN-030</t>
+          <t>MA10</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2192,7 +2236,7 @@
         </is>
       </c>
       <c r="D34" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E34" s="7" t="n">
         <v>2025</v>
@@ -2217,11 +2261,12 @@
       <c r="W34" s="8" t="n"/>
       <c r="X34" s="8" t="n"/>
       <c r="Y34" s="8" t="n"/>
+      <c r="Z34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>CEN-031</t>
+          <t>MA11</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -2235,7 +2280,7 @@
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>2025</v>
@@ -2260,16 +2305,17 @@
       <c r="W35" s="8" t="n"/>
       <c r="X35" s="8" t="n"/>
       <c r="Y35" s="8" t="n"/>
+      <c r="Z35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>CEN-032</t>
+          <t>NU1</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Ambagamuwa</t>
+          <t>Ambagamuwa Korale</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -2278,7 +2324,7 @@
         </is>
       </c>
       <c r="D36" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>2025</v>
@@ -2303,11 +2349,12 @@
       <c r="W36" s="8" t="n"/>
       <c r="X36" s="8" t="n"/>
       <c r="Y36" s="8" t="n"/>
+      <c r="Z36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>CEN-033</t>
+          <t>NU2</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2321,7 +2368,7 @@
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>2025</v>
@@ -2346,16 +2393,17 @@
       <c r="W37" s="8" t="n"/>
       <c r="X37" s="8" t="n"/>
       <c r="Y37" s="8" t="n"/>
+      <c r="Z37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>CEN-034</t>
+          <t>NU3</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Kothmale</t>
+          <t>Kothmale East</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -2364,7 +2412,7 @@
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>2025</v>
@@ -2389,25 +2437,26 @@
       <c r="W38" s="8" t="n"/>
       <c r="X38" s="8" t="n"/>
       <c r="Y38" s="8" t="n"/>
+      <c r="Z38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>CEN-035</t>
+          <t>NU4</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
+          <t>Kothmale West</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
           <t>Nuwara Eliya</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Nuwara Eliya</t>
-        </is>
-      </c>
       <c r="D39" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>2025</v>
@@ -2432,16 +2481,17 @@
       <c r="W39" s="8" t="n"/>
       <c r="X39" s="8" t="n"/>
       <c r="Y39" s="8" t="n"/>
+      <c r="Z39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>CEN-036</t>
+          <t>NU5</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Walapane</t>
+          <t>Mathurata</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -2450,7 +2500,7 @@
         </is>
       </c>
       <c r="D40" s="7" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E40" s="7" t="n">
         <v>2025</v>
@@ -2475,14 +2525,234 @@
       <c r="W40" s="8" t="n"/>
       <c r="X40" s="8" t="n"/>
       <c r="Y40" s="8" t="n"/>
+      <c r="Z40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>NU6</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Nildandahinna</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
+      <c r="L41" s="8" t="n"/>
+      <c r="M41" s="8" t="n"/>
+      <c r="N41" s="8" t="n"/>
+      <c r="O41" s="8" t="n"/>
+      <c r="P41" s="8" t="n"/>
+      <c r="Q41" s="8" t="n"/>
+      <c r="R41" s="8" t="n"/>
+      <c r="S41" s="8" t="n"/>
+      <c r="T41" s="8" t="n"/>
+      <c r="U41" s="8" t="n"/>
+      <c r="V41" s="8" t="n"/>
+      <c r="W41" s="8" t="n"/>
+      <c r="X41" s="8" t="n"/>
+      <c r="Y41" s="8" t="n"/>
+      <c r="Z41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>NU7</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Norwood</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
+      <c r="L42" s="8" t="n"/>
+      <c r="M42" s="8" t="n"/>
+      <c r="N42" s="8" t="n"/>
+      <c r="O42" s="8" t="n"/>
+      <c r="P42" s="8" t="n"/>
+      <c r="Q42" s="8" t="n"/>
+      <c r="R42" s="8" t="n"/>
+      <c r="S42" s="8" t="n"/>
+      <c r="T42" s="8" t="n"/>
+      <c r="U42" s="8" t="n"/>
+      <c r="V42" s="8" t="n"/>
+      <c r="W42" s="8" t="n"/>
+      <c r="X42" s="8" t="n"/>
+      <c r="Y42" s="8" t="n"/>
+      <c r="Z42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>NU8</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+      <c r="K43" s="8" t="n"/>
+      <c r="L43" s="8" t="n"/>
+      <c r="M43" s="8" t="n"/>
+      <c r="N43" s="8" t="n"/>
+      <c r="O43" s="8" t="n"/>
+      <c r="P43" s="8" t="n"/>
+      <c r="Q43" s="8" t="n"/>
+      <c r="R43" s="8" t="n"/>
+      <c r="S43" s="8" t="n"/>
+      <c r="T43" s="8" t="n"/>
+      <c r="U43" s="8" t="n"/>
+      <c r="V43" s="8" t="n"/>
+      <c r="W43" s="8" t="n"/>
+      <c r="X43" s="8" t="n"/>
+      <c r="Y43" s="8" t="n"/>
+      <c r="Z43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>NU9</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Thalawakele</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+      <c r="K44" s="8" t="n"/>
+      <c r="L44" s="8" t="n"/>
+      <c r="M44" s="8" t="n"/>
+      <c r="N44" s="8" t="n"/>
+      <c r="O44" s="8" t="n"/>
+      <c r="P44" s="8" t="n"/>
+      <c r="Q44" s="8" t="n"/>
+      <c r="R44" s="8" t="n"/>
+      <c r="S44" s="8" t="n"/>
+      <c r="T44" s="8" t="n"/>
+      <c r="U44" s="8" t="n"/>
+      <c r="V44" s="8" t="n"/>
+      <c r="W44" s="8" t="n"/>
+      <c r="X44" s="8" t="n"/>
+      <c r="Y44" s="8" t="n"/>
+      <c r="Z44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>NU10</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Walapane</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="n"/>
+      <c r="H45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8" t="n"/>
+      <c r="K45" s="8" t="n"/>
+      <c r="L45" s="8" t="n"/>
+      <c r="M45" s="8" t="n"/>
+      <c r="N45" s="8" t="n"/>
+      <c r="O45" s="8" t="n"/>
+      <c r="P45" s="8" t="n"/>
+      <c r="Q45" s="8" t="n"/>
+      <c r="R45" s="8" t="n"/>
+      <c r="S45" s="8" t="n"/>
+      <c r="T45" s="8" t="n"/>
+      <c r="U45" s="8" t="n"/>
+      <c r="V45" s="8" t="n"/>
+      <c r="W45" s="8" t="n"/>
+      <c r="X45" s="8" t="n"/>
+      <c r="Y45" s="8" t="n"/>
+      <c r="Z45" s="8" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 P5 P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 S40 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T16 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T27 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 V5 V6 V7 V8 V9 V10 V11 V12 V13 V14 V15 V16 V17 V18 V19 V20 V21 V22 V23 V24 V25 V26 V27 V28 V29 V30 V31 V32 V33 V34 V35 V36 V37 V38 V39 V40 W5 W6 W7 W8 W9 W10 W11 W12 W13 W14 W15 W16 W17 W18 W19 W20 W21 W22 W23 W24 W25 W26 W27 W28 W29 W30 W31 W32 W33 W34 W35 W36 W37 W38 W39 W40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Raw values must be numbers &gt;= 0." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 M41 M42 M43 M44 M45 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 P5 P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 P41 P42 P43 P44 P45 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 S40 S41 S42 S43 S44 S45 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T16 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T27 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 T41 T42 T43 T44 T45 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 V5 V6 V7 V8 V9 V10 V11 V12 V13 V14 V15 V16 V17 V18 V19 V20 V21 V22 V23 V24 V25 V26 V27 V28 V29 V30 V31 V32 V33 V34 V35 V36 V37 V38 V39 V40 V41 V42 V43 V44 V45 W5 W6 W7 W8 W9 W10 W11 W12 W13 W14 W15 W16 W17 W18 W19 W20 W21 W22 W23 W24 W25 W26 W27 W28 W29 W30 W31 W32 W33 W34 W35 W36 W37 W38 W39 W40 W41 W42 W43 W44 W45 X5 X6 X7 X8 X9 X10 X11 X12 X13 X14 X15 X16 X17 X18 X19 X20 X21 X22 X23 X24 X25 X26 X27 X28 X29 X30 X31 X32 X33 X34 X35 X36 X37 X38 X39 X40 X41 X42 X43 X44 X45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Raw values must be numbers &gt;= 0." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2496,7 +2766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y40"/>
+  <dimension ref="A1:Z45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2524,12 +2794,13 @@
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="16" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RAW DATA 2025-2030 - Livestock Sector / Buffalo Farming - Drought - Central Province   [profile BUFFALO_DROUGHT_CEN_V1]   |   Enter RAW values only - the system normalizes.</t>
+          <t>RAW DATA 2026-2030 - Livestock Sector / Buffalo Farming - Drought - Central Province   [profile BUFFALO_DROUGHT_CEN_V1]   |   Enter RAW values only - the system normalizes.</t>
         </is>
       </c>
     </row>
@@ -2561,100 +2832,105 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>DROUGHT_EVENTS_1974_TO_2022</t>
+          <t>DROUGHT_EVENTS_1974_TO_2004</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>DROUGHT_EVENTS_2005_TO_2022</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
           <t>DROUGHT_HAZARD_INDEX</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>OCCURRENCE_WARM_DAYS</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>STANDARD_PRECIPITATION_INDEX</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_FARMERS</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_FARMS</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_MILK_PRODUCTION_FARMS</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>BUFFALO_POPULATION</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>LIVESTOCK_FARMERS</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>MITCH_BUFFALOES_DAILY_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>PASTURE_FODDER_EXTENT_ACRE</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>PCT_EXTENSIVE</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>PCT_INTENSIVE</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>PCT_SEMI_INTENSIVE</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="Y2" s="2" t="inlineStr">
         <is>
           <t>DATA_SOURCE</t>
         </is>
       </c>
-      <c r="Y2" s="2" t="inlineStr">
+      <c r="Z2" s="2" t="inlineStr">
         <is>
           <t>NOTES</t>
         </is>
@@ -2688,118 +2964,124 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>hazard: No. of drought events - 1974 to 2022 (1974-2004, 25%, 2005 -2022, 75%)
-&gt;&gt; fixed window - same value on both period tabs</t>
+          <t>hazard: No. of Drought events - 1974 to 2004 (25%)
+&gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>hazard: No. of Drought events - 2005 -2022 (75%)
+&gt;&gt; enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>hazard: Drought Hazard  Index
 &gt;&gt; fixed window - same value on both period tabs</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>hazard: Occurrence of warm days (TX90p)
 &gt;&gt; fixed window - same value on both period tabs</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>hazard: SPI (Intensity)
 &gt;&gt; fixed window - same value on both period tabs</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>exposure: # of Buffalo Farmers
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>exposure: No. of Buffalo Farms
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>exposure: No.of Buffalo Milk Production Farms
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>exposure: Buffalo Population
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>exposure: Total livestock farmers
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>exposure: Annual Mitch Buffalo Milk Production (l)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>exposure: Daily Mitch Buffaloes Milk Production (l)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>exposure: Mitch Buffalo Monthly Milk Production (l)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>exposure: Pasture &amp; Fodder Extent (Acre)
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>exposure: % of Buffalo Farmers from total livestock operators
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>exposure: % Extensive
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr">
+      <c r="V3" s="5" t="inlineStr">
         <is>
           <t>exposure: % Intensive
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="V3" s="5" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr">
         <is>
           <t>exposure: % livestock farmers from total Agricultural Operators
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr">
+      <c r="X3" s="5" t="inlineStr">
         <is>
           <t>exposure: % Semi Intensive
 &gt;&gt; enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
-      <c r="X3" s="5" t="inlineStr">
+      <c r="Y3" s="5" t="inlineStr">
         <is>
           <t>origin of the numbers</t>
         </is>
       </c>
-      <c r="Y3" s="5" t="inlineStr">
+      <c r="Z3" s="5" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
@@ -2822,7 +3104,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E4" s="6" t="n">
         <v>2030</v>
@@ -2881,12 +3163,15 @@
       <c r="W4" s="6" t="n">
         <v>737.5</v>
       </c>
-      <c r="X4" s="6" t="inlineStr">
-        <is>
-          <t>Dept. report 2025-2030</t>
-        </is>
+      <c r="X4" s="6" t="n">
+        <v>775</v>
       </c>
       <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>Dept. report 2026-2030</t>
+        </is>
+      </c>
+      <c r="Z4" s="6" t="inlineStr">
         <is>
           <t>example row</t>
         </is>
@@ -2895,7 +3180,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>CEN-001</t>
+          <t>KA1</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -2909,7 +3194,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>2030</v>
@@ -2934,11 +3219,12 @@
       <c r="W5" s="8" t="n"/>
       <c r="X5" s="8" t="n"/>
       <c r="Y5" s="8" t="n"/>
+      <c r="Z5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>CEN-002</t>
+          <t>KA2</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -2952,7 +3238,7 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>2030</v>
@@ -2977,11 +3263,12 @@
       <c r="W6" s="8" t="n"/>
       <c r="X6" s="8" t="n"/>
       <c r="Y6" s="8" t="n"/>
+      <c r="Z6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>CEN-003</t>
+          <t>KA3</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -2995,7 +3282,7 @@
         </is>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>2030</v>
@@ -3020,11 +3307,12 @@
       <c r="W7" s="8" t="n"/>
       <c r="X7" s="8" t="n"/>
       <c r="Y7" s="8" t="n"/>
+      <c r="Z7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>CEN-004</t>
+          <t>KA4</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -3038,7 +3326,7 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>2030</v>
@@ -3063,11 +3351,12 @@
       <c r="W8" s="8" t="n"/>
       <c r="X8" s="8" t="n"/>
       <c r="Y8" s="8" t="n"/>
+      <c r="Z8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>CEN-005</t>
+          <t>KA5</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -3081,7 +3370,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>2030</v>
@@ -3106,11 +3395,12 @@
       <c r="W9" s="8" t="n"/>
       <c r="X9" s="8" t="n"/>
       <c r="Y9" s="8" t="n"/>
+      <c r="Z9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>CEN-006</t>
+          <t>KA6</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -3124,7 +3414,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>2030</v>
@@ -3149,11 +3439,12 @@
       <c r="W10" s="8" t="n"/>
       <c r="X10" s="8" t="n"/>
       <c r="Y10" s="8" t="n"/>
+      <c r="Z10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>CEN-007</t>
+          <t>KA7</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -3167,7 +3458,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>2030</v>
@@ -3192,11 +3483,12 @@
       <c r="W11" s="8" t="n"/>
       <c r="X11" s="8" t="n"/>
       <c r="Y11" s="8" t="n"/>
+      <c r="Z11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>CEN-008</t>
+          <t>KA8</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -3210,7 +3502,7 @@
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>2030</v>
@@ -3235,11 +3527,12 @@
       <c r="W12" s="8" t="n"/>
       <c r="X12" s="8" t="n"/>
       <c r="Y12" s="8" t="n"/>
+      <c r="Z12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>CEN-009</t>
+          <t>KA9</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -3253,7 +3546,7 @@
         </is>
       </c>
       <c r="D13" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>2030</v>
@@ -3278,11 +3571,12 @@
       <c r="W13" s="8" t="n"/>
       <c r="X13" s="8" t="n"/>
       <c r="Y13" s="8" t="n"/>
+      <c r="Z13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>CEN-010</t>
+          <t>KA10</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -3296,7 +3590,7 @@
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>2030</v>
@@ -3321,11 +3615,12 @@
       <c r="W14" s="8" t="n"/>
       <c r="X14" s="8" t="n"/>
       <c r="Y14" s="8" t="n"/>
+      <c r="Z14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>CEN-011</t>
+          <t>KA11</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -3339,7 +3634,7 @@
         </is>
       </c>
       <c r="D15" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>2030</v>
@@ -3364,11 +3659,12 @@
       <c r="W15" s="8" t="n"/>
       <c r="X15" s="8" t="n"/>
       <c r="Y15" s="8" t="n"/>
+      <c r="Z15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>CEN-012</t>
+          <t>KA12</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -3382,7 +3678,7 @@
         </is>
       </c>
       <c r="D16" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>2030</v>
@@ -3407,11 +3703,12 @@
       <c r="W16" s="8" t="n"/>
       <c r="X16" s="8" t="n"/>
       <c r="Y16" s="8" t="n"/>
+      <c r="Z16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>CEN-013</t>
+          <t>KA13</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -3425,7 +3722,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>2030</v>
@@ -3450,11 +3747,12 @@
       <c r="W17" s="8" t="n"/>
       <c r="X17" s="8" t="n"/>
       <c r="Y17" s="8" t="n"/>
+      <c r="Z17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>CEN-014</t>
+          <t>KA14</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -3468,7 +3766,7 @@
         </is>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>2030</v>
@@ -3493,11 +3791,12 @@
       <c r="W18" s="8" t="n"/>
       <c r="X18" s="8" t="n"/>
       <c r="Y18" s="8" t="n"/>
+      <c r="Z18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>CEN-015</t>
+          <t>KA15</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -3511,7 +3810,7 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>2030</v>
@@ -3536,11 +3835,12 @@
       <c r="W19" s="8" t="n"/>
       <c r="X19" s="8" t="n"/>
       <c r="Y19" s="8" t="n"/>
+      <c r="Z19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>CEN-016</t>
+          <t>KA16</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -3554,7 +3854,7 @@
         </is>
       </c>
       <c r="D20" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>2030</v>
@@ -3579,11 +3879,12 @@
       <c r="W20" s="8" t="n"/>
       <c r="X20" s="8" t="n"/>
       <c r="Y20" s="8" t="n"/>
+      <c r="Z20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>CEN-017</t>
+          <t>KA17</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -3597,7 +3898,7 @@
         </is>
       </c>
       <c r="D21" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E21" s="7" t="n">
         <v>2030</v>
@@ -3622,11 +3923,12 @@
       <c r="W21" s="8" t="n"/>
       <c r="X21" s="8" t="n"/>
       <c r="Y21" s="8" t="n"/>
+      <c r="Z21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>CEN-018</t>
+          <t>KA18</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -3640,7 +3942,7 @@
         </is>
       </c>
       <c r="D22" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E22" s="7" t="n">
         <v>2030</v>
@@ -3665,11 +3967,12 @@
       <c r="W22" s="8" t="n"/>
       <c r="X22" s="8" t="n"/>
       <c r="Y22" s="8" t="n"/>
+      <c r="Z22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>CEN-019</t>
+          <t>KA19</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -3683,7 +3986,7 @@
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>2030</v>
@@ -3708,11 +4011,12 @@
       <c r="W23" s="8" t="n"/>
       <c r="X23" s="8" t="n"/>
       <c r="Y23" s="8" t="n"/>
+      <c r="Z23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>CEN-020</t>
+          <t>KA20</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -3726,7 +4030,7 @@
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>2030</v>
@@ -3751,11 +4055,12 @@
       <c r="W24" s="8" t="n"/>
       <c r="X24" s="8" t="n"/>
       <c r="Y24" s="8" t="n"/>
+      <c r="Z24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>CEN-021</t>
+          <t>MA1</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -3769,7 +4074,7 @@
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>2030</v>
@@ -3794,11 +4099,12 @@
       <c r="W25" s="8" t="n"/>
       <c r="X25" s="8" t="n"/>
       <c r="Y25" s="8" t="n"/>
+      <c r="Z25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>CEN-022</t>
+          <t>MA2</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -3812,7 +4118,7 @@
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>2030</v>
@@ -3837,11 +4143,12 @@
       <c r="W26" s="8" t="n"/>
       <c r="X26" s="8" t="n"/>
       <c r="Y26" s="8" t="n"/>
+      <c r="Z26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>CEN-023</t>
+          <t>MA3</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -3855,7 +4162,7 @@
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>2030</v>
@@ -3880,11 +4187,12 @@
       <c r="W27" s="8" t="n"/>
       <c r="X27" s="8" t="n"/>
       <c r="Y27" s="8" t="n"/>
+      <c r="Z27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>CEN-024</t>
+          <t>MA4</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -3898,7 +4206,7 @@
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>2030</v>
@@ -3923,11 +4231,12 @@
       <c r="W28" s="8" t="n"/>
       <c r="X28" s="8" t="n"/>
       <c r="Y28" s="8" t="n"/>
+      <c r="Z28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>CEN-025</t>
+          <t>MA5</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -3941,7 +4250,7 @@
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E29" s="7" t="n">
         <v>2030</v>
@@ -3966,11 +4275,12 @@
       <c r="W29" s="8" t="n"/>
       <c r="X29" s="8" t="n"/>
       <c r="Y29" s="8" t="n"/>
+      <c r="Z29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>CEN-026</t>
+          <t>MA6</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -3984,7 +4294,7 @@
         </is>
       </c>
       <c r="D30" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E30" s="7" t="n">
         <v>2030</v>
@@ -4009,11 +4319,12 @@
       <c r="W30" s="8" t="n"/>
       <c r="X30" s="8" t="n"/>
       <c r="Y30" s="8" t="n"/>
+      <c r="Z30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>CEN-027</t>
+          <t>MA7</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -4027,7 +4338,7 @@
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>2030</v>
@@ -4052,11 +4363,12 @@
       <c r="W31" s="8" t="n"/>
       <c r="X31" s="8" t="n"/>
       <c r="Y31" s="8" t="n"/>
+      <c r="Z31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>CEN-028</t>
+          <t>MA8</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -4070,7 +4382,7 @@
         </is>
       </c>
       <c r="D32" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>2030</v>
@@ -4095,11 +4407,12 @@
       <c r="W32" s="8" t="n"/>
       <c r="X32" s="8" t="n"/>
       <c r="Y32" s="8" t="n"/>
+      <c r="Z32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>CEN-029</t>
+          <t>MA9</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -4113,7 +4426,7 @@
         </is>
       </c>
       <c r="D33" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E33" s="7" t="n">
         <v>2030</v>
@@ -4138,11 +4451,12 @@
       <c r="W33" s="8" t="n"/>
       <c r="X33" s="8" t="n"/>
       <c r="Y33" s="8" t="n"/>
+      <c r="Z33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>CEN-030</t>
+          <t>MA10</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -4156,7 +4470,7 @@
         </is>
       </c>
       <c r="D34" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E34" s="7" t="n">
         <v>2030</v>
@@ -4181,11 +4495,12 @@
       <c r="W34" s="8" t="n"/>
       <c r="X34" s="8" t="n"/>
       <c r="Y34" s="8" t="n"/>
+      <c r="Z34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>CEN-031</t>
+          <t>MA11</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -4199,7 +4514,7 @@
         </is>
       </c>
       <c r="D35" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>2030</v>
@@ -4224,16 +4539,17 @@
       <c r="W35" s="8" t="n"/>
       <c r="X35" s="8" t="n"/>
       <c r="Y35" s="8" t="n"/>
+      <c r="Z35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>CEN-032</t>
+          <t>NU1</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Ambagamuwa</t>
+          <t>Ambagamuwa Korale</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -4242,7 +4558,7 @@
         </is>
       </c>
       <c r="D36" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>2030</v>
@@ -4267,11 +4583,12 @@
       <c r="W36" s="8" t="n"/>
       <c r="X36" s="8" t="n"/>
       <c r="Y36" s="8" t="n"/>
+      <c r="Z36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>CEN-033</t>
+          <t>NU2</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -4285,7 +4602,7 @@
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E37" s="7" t="n">
         <v>2030</v>
@@ -4310,16 +4627,17 @@
       <c r="W37" s="8" t="n"/>
       <c r="X37" s="8" t="n"/>
       <c r="Y37" s="8" t="n"/>
+      <c r="Z37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>CEN-034</t>
+          <t>NU3</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Kothmale</t>
+          <t>Kothmale East</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -4328,7 +4646,7 @@
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>2030</v>
@@ -4353,25 +4671,26 @@
       <c r="W38" s="8" t="n"/>
       <c r="X38" s="8" t="n"/>
       <c r="Y38" s="8" t="n"/>
+      <c r="Z38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>CEN-035</t>
+          <t>NU4</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
+          <t>Kothmale West</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
           <t>Nuwara Eliya</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Nuwara Eliya</t>
-        </is>
-      </c>
       <c r="D39" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>2030</v>
@@ -4396,16 +4715,17 @@
       <c r="W39" s="8" t="n"/>
       <c r="X39" s="8" t="n"/>
       <c r="Y39" s="8" t="n"/>
+      <c r="Z39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>CEN-036</t>
+          <t>NU5</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Walapane</t>
+          <t>Mathurata</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -4414,7 +4734,7 @@
         </is>
       </c>
       <c r="D40" s="7" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E40" s="7" t="n">
         <v>2030</v>
@@ -4439,14 +4759,234 @@
       <c r="W40" s="8" t="n"/>
       <c r="X40" s="8" t="n"/>
       <c r="Y40" s="8" t="n"/>
+      <c r="Z40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>NU6</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Nildandahinna</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>2030</v>
+      </c>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
+      <c r="L41" s="8" t="n"/>
+      <c r="M41" s="8" t="n"/>
+      <c r="N41" s="8" t="n"/>
+      <c r="O41" s="8" t="n"/>
+      <c r="P41" s="8" t="n"/>
+      <c r="Q41" s="8" t="n"/>
+      <c r="R41" s="8" t="n"/>
+      <c r="S41" s="8" t="n"/>
+      <c r="T41" s="8" t="n"/>
+      <c r="U41" s="8" t="n"/>
+      <c r="V41" s="8" t="n"/>
+      <c r="W41" s="8" t="n"/>
+      <c r="X41" s="8" t="n"/>
+      <c r="Y41" s="8" t="n"/>
+      <c r="Z41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>NU7</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Norwood</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>2030</v>
+      </c>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
+      <c r="L42" s="8" t="n"/>
+      <c r="M42" s="8" t="n"/>
+      <c r="N42" s="8" t="n"/>
+      <c r="O42" s="8" t="n"/>
+      <c r="P42" s="8" t="n"/>
+      <c r="Q42" s="8" t="n"/>
+      <c r="R42" s="8" t="n"/>
+      <c r="S42" s="8" t="n"/>
+      <c r="T42" s="8" t="n"/>
+      <c r="U42" s="8" t="n"/>
+      <c r="V42" s="8" t="n"/>
+      <c r="W42" s="8" t="n"/>
+      <c r="X42" s="8" t="n"/>
+      <c r="Y42" s="8" t="n"/>
+      <c r="Z42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>NU8</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>2030</v>
+      </c>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+      <c r="K43" s="8" t="n"/>
+      <c r="L43" s="8" t="n"/>
+      <c r="M43" s="8" t="n"/>
+      <c r="N43" s="8" t="n"/>
+      <c r="O43" s="8" t="n"/>
+      <c r="P43" s="8" t="n"/>
+      <c r="Q43" s="8" t="n"/>
+      <c r="R43" s="8" t="n"/>
+      <c r="S43" s="8" t="n"/>
+      <c r="T43" s="8" t="n"/>
+      <c r="U43" s="8" t="n"/>
+      <c r="V43" s="8" t="n"/>
+      <c r="W43" s="8" t="n"/>
+      <c r="X43" s="8" t="n"/>
+      <c r="Y43" s="8" t="n"/>
+      <c r="Z43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>NU9</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Thalawakele</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>2030</v>
+      </c>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+      <c r="K44" s="8" t="n"/>
+      <c r="L44" s="8" t="n"/>
+      <c r="M44" s="8" t="n"/>
+      <c r="N44" s="8" t="n"/>
+      <c r="O44" s="8" t="n"/>
+      <c r="P44" s="8" t="n"/>
+      <c r="Q44" s="8" t="n"/>
+      <c r="R44" s="8" t="n"/>
+      <c r="S44" s="8" t="n"/>
+      <c r="T44" s="8" t="n"/>
+      <c r="U44" s="8" t="n"/>
+      <c r="V44" s="8" t="n"/>
+      <c r="W44" s="8" t="n"/>
+      <c r="X44" s="8" t="n"/>
+      <c r="Y44" s="8" t="n"/>
+      <c r="Z44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>NU10</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Walapane</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Nuwara Eliya</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>2030</v>
+      </c>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="n"/>
+      <c r="H45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8" t="n"/>
+      <c r="K45" s="8" t="n"/>
+      <c r="L45" s="8" t="n"/>
+      <c r="M45" s="8" t="n"/>
+      <c r="N45" s="8" t="n"/>
+      <c r="O45" s="8" t="n"/>
+      <c r="P45" s="8" t="n"/>
+      <c r="Q45" s="8" t="n"/>
+      <c r="R45" s="8" t="n"/>
+      <c r="S45" s="8" t="n"/>
+      <c r="T45" s="8" t="n"/>
+      <c r="U45" s="8" t="n"/>
+      <c r="V45" s="8" t="n"/>
+      <c r="W45" s="8" t="n"/>
+      <c r="X45" s="8" t="n"/>
+      <c r="Y45" s="8" t="n"/>
+      <c r="Z45" s="8" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A1:Z1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 P5 P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 S40 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T16 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T27 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 V5 V6 V7 V8 V9 V10 V11 V12 V13 V14 V15 V16 V17 V18 V19 V20 V21 V22 V23 V24 V25 V26 V27 V28 V29 V30 V31 V32 V33 V34 V35 V36 V37 V38 V39 V40 W5 W6 W7 W8 W9 W10 W11 W12 W13 W14 W15 W16 W17 W18 W19 W20 W21 W22 W23 W24 W25 W26 W27 W28 W29 W30 W31 W32 W33 W34 W35 W36 W37 W38 W39 W40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Raw values must be numbers &gt;= 0." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 I5 I6 I7 I8 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20 I21 I22 I23 I24 I25 I26 I27 I28 I29 I30 I31 I32 I33 I34 I35 I36 I37 I38 I39 I40 I41 I42 I43 I44 I45 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 L5 L6 L7 L8 L9 L10 L11 L12 L13 L14 L15 L16 L17 L18 L19 L20 L21 L22 L23 L24 L25 L26 L27 L28 L29 L30 L31 L32 L33 L34 L35 L36 L37 L38 L39 L40 L41 L42 L43 L44 L45 M5 M6 M7 M8 M9 M10 M11 M12 M13 M14 M15 M16 M17 M18 M19 M20 M21 M22 M23 M24 M25 M26 M27 M28 M29 M30 M31 M32 M33 M34 M35 M36 M37 M38 M39 M40 M41 M42 M43 M44 M45 N5 N6 N7 N8 N9 N10 N11 N12 N13 N14 N15 N16 N17 N18 N19 N20 N21 N22 N23 N24 N25 N26 N27 N28 N29 N30 N31 N32 N33 N34 N35 N36 N37 N38 N39 N40 N41 N42 N43 N44 N45 O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 P5 P6 P7 P8 P9 P10 P11 P12 P13 P14 P15 P16 P17 P18 P19 P20 P21 P22 P23 P24 P25 P26 P27 P28 P29 P30 P31 P32 P33 P34 P35 P36 P37 P38 P39 P40 P41 P42 P43 P44 P45 Q5 Q6 Q7 Q8 Q9 Q10 Q11 Q12 Q13 Q14 Q15 Q16 Q17 Q18 Q19 Q20 Q21 Q22 Q23 Q24 Q25 Q26 Q27 Q28 Q29 Q30 Q31 Q32 Q33 Q34 Q35 Q36 Q37 Q38 Q39 Q40 Q41 Q42 Q43 Q44 Q45 R5 R6 R7 R8 R9 R10 R11 R12 R13 R14 R15 R16 R17 R18 R19 R20 R21 R22 R23 R24 R25 R26 R27 R28 R29 R30 R31 R32 R33 R34 R35 R36 R37 R38 R39 R40 R41 R42 R43 R44 R45 S5 S6 S7 S8 S9 S10 S11 S12 S13 S14 S15 S16 S17 S18 S19 S20 S21 S22 S23 S24 S25 S26 S27 S28 S29 S30 S31 S32 S33 S34 S35 S36 S37 S38 S39 S40 S41 S42 S43 S44 S45 T5 T6 T7 T8 T9 T10 T11 T12 T13 T14 T15 T16 T17 T18 T19 T20 T21 T22 T23 T24 T25 T26 T27 T28 T29 T30 T31 T32 T33 T34 T35 T36 T37 T38 T39 T40 T41 T42 T43 T44 T45 U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 V5 V6 V7 V8 V9 V10 V11 V12 V13 V14 V15 V16 V17 V18 V19 V20 V21 V22 V23 V24 V25 V26 V27 V28 V29 V30 V31 V32 V33 V34 V35 V36 V37 V38 V39 V40 V41 V42 V43 V44 V45 W5 W6 W7 W8 W9 W10 W11 W12 W13 W14 W15 W16 W17 W18 W19 W20 W21 W22 W23 W24 W25 W26 W27 W28 W29 W30 W31 W32 W33 W34 W35 W36 W37 W38 W39 W40 W41 W42 W43 W44 W45 X5 X6 X7 X8 X9 X10 X11 X12 X13 X14 X15 X16 X17 X18 X19 X20 X21 X22 X23 X24 X25 X26 X27 X28 X29 X30 X31 X32 X33 X34 X35 X36 X37 X38 X39 X40 X41 X42 X43 X44 X45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Raw values must be numbers &gt;= 0." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4460,7 +5000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4469,6 +5009,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4516,16 +5057,21 @@
           <t>PROPOSED WEIGHT % (read at import)</t>
         </is>
       </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>basis of the proposal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>DROUGHT_EVENTS_1974_TO_2022</t>
+          <t>DROUGHT_EVENTS_1974_TO_2004</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>No. of drought events - 1974 to 2022 (1974-2004, 25%, 2005 -2022, 75%)</t>
+          <t>No. of Drought events - 1974 to 2004 (25%)</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -4533,171 +5079,182 @@
           <t>hazard</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>40</v>
-      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
       <c r="F4" s="12" t="n">
-        <v>40</v>
+        <v>10</v>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>derived: 25% of retired DROUGHT_EVENTS_1974_TO_2022 (40)</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>DROUGHT_HAZARD_INDEX</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Drought Hazard  Index</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>DROUGHT_EVENTS_2005_TO_2022</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>No. of Drought events - 2005 -2022 (75%)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>hazard</t>
         </is>
       </c>
-      <c r="D5" s="13" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="12" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>derived: 75% of retired DROUGHT_EVENTS_1974_TO_2022 (40)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
+          <t>DROUGHT_HAZARD_INDEX</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Drought Hazard  Index</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>hazard</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
           <t>OCCURRENCE_WARM_DAYS</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Occurrence of warm days (TX90p)</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>hazard</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E7" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F7" s="12" t="n">
         <v>15</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>STANDARD_PRECIPITATION_INDEX</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>SPI (Intensity)</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>hazard</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E8" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F8" s="12" t="n">
         <v>45</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>BUFFALO_FARMERS</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t># of Buffalo Farmers</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>20</v>
-      </c>
+      <c r="G8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
+          <t>BUFFALO_FARMERS</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t># of Buffalo Farmers</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
           <t>BUFFALO_FARMS</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>No. of Buffalo Farms</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="12" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>BUFFALO_MILK_PRODUCTION_FARMS</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>No.of Buffalo Milk Production Farms</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
       <c r="F10" s="12" t="n"/>
+      <c r="G10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>BUFFALO_POPULATION</t>
+          <t>BUFFALO_MILK_PRODUCTION_FARMS</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Buffalo Population</t>
+          <t>No.of Buffalo Milk Production Farms</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -4705,27 +5262,20 @@
           <t>exposure</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>20</v>
-      </c>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>LIVESTOCK_FARMERS</t>
+          <t>BUFFALO_POPULATION</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Total livestock farmers</t>
+          <t>Buffalo Population</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -4733,19 +5283,28 @@
           <t>exposure</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="12" t="n"/>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION</t>
+          <t>LIVESTOCK_FARMERS</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Annual Mitch Buffalo Milk Production (l)</t>
+          <t>Total livestock farmers</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -4753,223 +5312,252 @@
           <t>exposure</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>40</v>
-      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
+          <t>MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Annual Mitch Buffalo Milk Production (l)</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
           <t>MITCH_BUFFALOES_DAILY_MILK_PRODUCTION</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Daily Mitch Buffaloes Milk Production (l)</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="12" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Mitch Buffalo Monthly Milk Production (l)</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
       <c r="F15" s="12" t="n"/>
+      <c r="G15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
+          <t>MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Mitch Buffalo Monthly Milk Production (l)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
           <t>PASTURE_FODDER_EXTENT_ACRE</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Pasture &amp; Fodder Extent (Acre)</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="F16" s="12" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>% of Buffalo Farmers from total livestock operators</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="13" t="n">
         <v>10</v>
       </c>
       <c r="F17" s="12" t="n">
         <v>10</v>
       </c>
+      <c r="G17" s="13" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
         <is>
+          <t>PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>% of Buffalo Farmers from total livestock operators</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
           <t>PCT_EXTENSIVE</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>% Extensive</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="12" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>PCT_INTENSIVE</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>% Intensive</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="12" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>% livestock farmers from total Agricultural Operators</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="12" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="11" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>PCT_SEMI_INTENSIVE</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>% Semi Intensive</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="12" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>SUM - hazard (must equal 100)</t>
-        </is>
-      </c>
-      <c r="F23" s="15">
-        <f>F4+F5+F6+F7</f>
-        <v/>
-      </c>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
+          <t>SUM - hazard (must equal 100)</t>
+        </is>
+      </c>
+      <c r="F24" s="15">
+        <f>F4+F5+F6+F7+F8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
           <t>SUM - exposure (must equal 100)</t>
         </is>
       </c>
-      <c r="F24" s="15">
-        <f>F8+F9+F10+F11+F12+F13+F14+F15+F16+F17+F18+F19+F20+F21</f>
+      <c r="F25" s="15">
+        <f>F9+F10+F11+F12+F13+F14+F15+F16+F17+F18+F19+F20+F21+F22</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid weight" error="Weight must be between 0 and 100." type="decimal" operator="between">
+    <dataValidation sqref="F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid weight" error="Weight must be between 0 and 100." type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
@@ -4984,7 +5572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5005,14 +5593,14 @@
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Profile: BUFFALO_DROUGHT_CEN_V1   |   generated 2026-07-29 from FINAL_VARIABLES.xlsx (expert-refined catalog)</t>
+          <t>Profile: BUFFALO_DROUGHT_CEN_V1   |   generated 2026-09-03 from FINAL_VARIABLES.xlsx (expert-refined catalog)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>1. One tab per data period (2020-2025, 2025-2030). Fill the tab matching your dataset's period; skip tabs with no data.</t>
+          <t>1. One tab per data period (2021-2025, 2026-2030). Fill the tab matching your dataset's period; skip tabs with no data.</t>
         </is>
       </c>
     </row>
@@ -5026,14 +5614,14 @@
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>2b. The year 2025 appears in both tabs. If a year sits in two periods the system uses the LATER period's value, so nothing is counted twice.</t>
+          <t>2b. The two periods are contiguous and do not overlap (changed 2026-09-03 at the Central panel's request - the old 2020-2025 / 2025-2030 pair shared the year 2025 and needed a tie-break). Every year belongs to exactly one tab.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>3. Edit ONLY the yellow cells. Division codes, names, district and the period columns are pre-filled and locked.</t>
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>3. REVIEW COPY - nothing is locked. The yellow cells are still where data belongs, but every cell, header and tab can be changed so the panel can mark up structure as well as values. Return the marked-up file; the finalised version will be re-issued locked for collection.</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5635,7 @@
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>5. Do not add, remove, rename or reorder columns or tabs. Files with changed structure are rejected on import.</t>
+          <t>5. Structural changes ARE invited in this review copy - add, rename or reorder columns and note what you changed. This file is NOT importable; the locked re-issue is.</t>
         </is>
       </c>
     </row>
@@ -5119,480 +5707,498 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>DROUGHT_EVENTS_1974_TO_2022</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>No. of drought events - 1974 to 2022 (1974-2004, 25%, 2005 -2022, 75%)</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>DROUGHT_EVENTS_1974_TO_2004</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>No. of Drought events - 1974 to 2004 (25%)</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>hazard</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>DROUGHT_EVENTS_2005_TO_2022</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>No. of Drought events - 2005 -2022 (75%)</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>hazard</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>DROUGHT_HAZARD_INDEX</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Drought Hazard  Index</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>hazard</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>fixed window - same value on both period tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>OCCURRENCE_WARM_DAYS</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Occurrence of warm days (TX90p)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>hazard</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E21" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>fixed window - same value on both period tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>STANDARD_PRECIPITATION_INDEX</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>SPI (Intensity)</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>hazard</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>45</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>fixed window - same value on both period tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>BUFFALO_FARMERS</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t># of Buffalo Farmers</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>BUFFALO_FARMS</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>No. of Buffalo Farms</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>BUFFALO_MILK_PRODUCTION_FARMS</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>No.of Buffalo Milk Production Farms</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>BUFFALO_POPULATION</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Buffalo Population</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>LIVESTOCK_FARMERS</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Total livestock farmers</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Annual Mitch Buffalo Milk Production (l)</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>fixed window - same value on both period tabs</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>DROUGHT_HAZARD_INDEX</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Drought Hazard  Index</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>hazard</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>fixed window - same value on both period tabs</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>OCCURRENCE_WARM_DAYS</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Occurrence of warm days (TX90p)</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>hazard</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>MITCH_BUFFALOES_DAILY_MILK_PRODUCTION</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Daily Mitch Buffaloes Milk Production (l)</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Mitch Buffalo Monthly Milk Production (l)</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>PASTURE_FODDER_EXTENT_ACRE</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Pasture &amp; Fodder Extent (Acre)</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E20" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>fixed window - same value on both period tabs</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>STANDARD_PRECIPITATION_INDEX</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>SPI (Intensity)</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>hazard</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="E31" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>% of Buffalo Farmers from total livestock operators</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>exposure</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>45</v>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <t>fixed window - same value on both period tabs</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>BUFFALO_FARMERS</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t># of Buffalo Farmers</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="E32" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>enter a TYPICAL YEAR (not a total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>PCT_EXTENSIVE</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>% Extensive</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
+      <c r="D33" s="13" t="n"/>
+      <c r="E33" s="13" t="n"/>
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>BUFFALO_FARMS</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>No. of Buffalo Farms</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>PCT_INTENSIVE</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>% Intensive</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="D34" s="13" t="n"/>
+      <c r="E34" s="13" t="n"/>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>BUFFALO_MILK_PRODUCTION_FARMS</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>No.of Buffalo Milk Production Farms</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>% livestock farmers from total Agricultural Operators</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D24" s="11" t="n"/>
-      <c r="E24" s="11" t="n"/>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>enter a TYPICAL YEAR (not a total)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>BUFFALO_POPULATION</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Buffalo Population</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>PCT_SEMI_INTENSIVE</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>% Semi Intensive</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
         <is>
           <t>exposure</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>LIVESTOCK_FARMERS</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>Total livestock farmers</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="11" t="n"/>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Annual Mitch Buffalo Milk Production (l)</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>MITCH_BUFFALOES_DAILY_MILK_PRODUCTION</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Daily Mitch Buffaloes Milk Production (l)</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>Mitch Buffalo Monthly Milk Production (l)</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>PASTURE_FODDER_EXTENT_ACRE</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>Pasture &amp; Fodder Extent (Acre)</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="F30" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>% of Buffalo Farmers from total livestock operators</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>PCT_EXTENSIVE</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>% Extensive</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>PCT_INTENSIVE</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>% Intensive</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>% livestock farmers from total Agricultural Operators</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="n"/>
-      <c r="E34" s="11" t="n"/>
-      <c r="F34" s="11" t="inlineStr">
-        <is>
-          <t>enter a TYPICAL YEAR (not a total)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>PCT_SEMI_INTENSIVE</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="inlineStr">
-        <is>
-          <t>% Semi Intensive</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>exposure</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="11" t="inlineStr">
+      <c r="D36" s="13" t="n"/>
+      <c r="E36" s="13" t="n"/>
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>enter a TYPICAL YEAR (not a total)</t>
         </is>
@@ -5609,7 +6215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5697,82 +6303,106 @@
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>generated</t>
+          <t>protection</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>unlocked-review</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>dsd_level</t>
+          <t>panel_overrides</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>DS_DIVISION</t>
+          <t>2 add, 1 retire</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>periods</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>2020-2025|2025-2030</t>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>n_variables</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="n">
-        <v>18</v>
+          <t>dsd_level</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>DS_DIVISION</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>period_rule_default</t>
+          <t>periods</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>average (typical year); 2025 -&gt; latest period wins</t>
+          <t>2021-2025|2026-2030</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>period_aggregation</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>DROUGHT_EVENTS_1974_TO_2022=fixed_window|DROUGHT_HAZARD_INDEX=fixed_window|OCCURRENCE_WARM_DAYS=fixed_window|STANDARD_PRECIPITATION_INDEX=fixed_window|BUFFALO_FARMERS=average|BUFFALO_FARMS=average|BUFFALO_MILK_PRODUCTION_FARMS=average|BUFFALO_POPULATION=average|LIVESTOCK_FARMERS=average|MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION=average|MITCH_BUFFALOES_DAILY_MILK_PRODUCTION=average|MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION=average|PASTURE_FODDER_EXTENT_ACRE=average|PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS=average|PCT_EXTENSIVE=average|PCT_INTENSIVE=average|PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS=average|PCT_SEMI_INTENSIVE=average</t>
-        </is>
+          <t>n_variables</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
+          <t>period_rule_default</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>average (typical year); periods are contiguous, no overlap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>period_aggregation</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>DROUGHT_EVENTS_1974_TO_2004=average|DROUGHT_EVENTS_2005_TO_2022=average|DROUGHT_HAZARD_INDEX=fixed_window|OCCURRENCE_WARM_DAYS=fixed_window|STANDARD_PRECIPITATION_INDEX=fixed_window|BUFFALO_FARMERS=average|BUFFALO_FARMS=average|BUFFALO_MILK_PRODUCTION_FARMS=average|BUFFALO_POPULATION=average|LIVESTOCK_FARMERS=average|MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION=average|MITCH_BUFFALOES_DAILY_MILK_PRODUCTION=average|MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION=average|PASTURE_FODDER_EXTENT_ACRE=average|PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS=average|PCT_EXTENSIVE=average|PCT_INTENSIVE=average|PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS=average|PCT_SEMI_INTENSIVE=average</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
           <t>expected_columns</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>DS_CODE|DS_DIVISION|DISTRICT|YEAR_START|YEAR_END|DROUGHT_EVENTS_1974_TO_2022|DROUGHT_HAZARD_INDEX|OCCURRENCE_WARM_DAYS|STANDARD_PRECIPITATION_INDEX|BUFFALO_FARMERS|BUFFALO_FARMS|BUFFALO_MILK_PRODUCTION_FARMS|BUFFALO_POPULATION|LIVESTOCK_FARMERS|MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION|MITCH_BUFFALOES_DAILY_MILK_PRODUCTION|MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION|PASTURE_FODDER_EXTENT_ACRE|PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS|PCT_EXTENSIVE|PCT_INTENSIVE|PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS|PCT_SEMI_INTENSIVE|DATA_SOURCE|NOTES</t>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>DS_CODE|DS_DIVISION|DISTRICT|YEAR_START|YEAR_END|DROUGHT_EVENTS_1974_TO_2004|DROUGHT_EVENTS_2005_TO_2022|DROUGHT_HAZARD_INDEX|OCCURRENCE_WARM_DAYS|STANDARD_PRECIPITATION_INDEX|BUFFALO_FARMERS|BUFFALO_FARMS|BUFFALO_MILK_PRODUCTION_FARMS|BUFFALO_POPULATION|LIVESTOCK_FARMERS|MITCH_BUFFALOES_ANNUAL_MILK_PRODUCTION|MITCH_BUFFALOES_DAILY_MILK_PRODUCTION|MITCH_BUFFALOES_MONTHLY_MILK_PRODUCTION|PASTURE_FODDER_EXTENT_ACRE|PCT_BUFFALO_FARMERS_LIVESTOCK_OPERATORS|PCT_EXTENSIVE|PCT_INTENSIVE|PCT_LIVESTOCK_FARMERS_AGRICULTURAL_OPERATORS|PCT_SEMI_INTENSIVE|DATA_SOURCE|NOTES</t>
         </is>
       </c>
     </row>

</xml_diff>